<commit_message>
result analysis in excel
</commit_message>
<xml_diff>
--- a/peak_load_shaving.xlsx
+++ b/peak_load_shaving.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dirk\Desktop\MVS\dev\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dirkl\OneDrive\Desktop\ongoing_projects\MVS\dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B137B424-CD62-4ED2-B1F0-317981537038}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD79D7D8-B388-42A5-8891-3BBFC2EDE9C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15840" xr2:uid="{9B5FF7E0-96E7-42B4-A4F2-AD52E30335CB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{9B5FF7E0-96E7-42B4-A4F2-AD52E30335CB}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
+    <sheet name="potential" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
   <si>
     <t>Hour</t>
   </si>
@@ -84,6 +85,15 @@
   </si>
   <si>
     <t>max_power_out_2050</t>
+  </si>
+  <si>
+    <t>nsq</t>
+  </si>
+  <si>
+    <t>l2050</t>
+  </si>
+  <si>
+    <t>l2024</t>
   </si>
 </sst>
 </file>
@@ -154,15 +164,15 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -178,7 +188,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -495,9 +505,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{346AC5F8-1765-463A-ABED-4754E8829304}">
   <dimension ref="A1:Z154"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:26" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:26" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -568,7 +578,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -642,7 +652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -716,7 +726,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -790,7 +800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -864,7 +874,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -938,7 +948,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -1012,7 +1022,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -1086,7 +1096,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -1160,7 +1170,7 @@
         <v>3.3330000000000002</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -1234,7 +1244,7 @@
         <v>3.6669999999999998</v>
       </c>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -1308,7 +1318,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -1382,7 +1392,7 @@
         <v>4.3330000000000002</v>
       </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -1456,7 +1466,7 @@
         <v>4.6669999999999998</v>
       </c>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>12</v>
       </c>
@@ -1530,7 +1540,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>13</v>
       </c>
@@ -1604,7 +1614,7 @@
         <v>5.25</v>
       </c>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>14</v>
       </c>
@@ -1678,7 +1688,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>15</v>
       </c>
@@ -1752,7 +1762,7 @@
         <v>5.75</v>
       </c>
     </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>16</v>
       </c>
@@ -1826,7 +1836,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>17</v>
       </c>
@@ -1900,7 +1910,7 @@
         <v>6.25</v>
       </c>
     </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>18</v>
       </c>
@@ -1974,7 +1984,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>19</v>
       </c>
@@ -2048,7 +2058,7 @@
         <v>6.75</v>
       </c>
     </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>20</v>
       </c>
@@ -2122,7 +2132,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>21</v>
       </c>
@@ -2196,7 +2206,7 @@
         <v>7.1669999999999998</v>
       </c>
     </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>22</v>
       </c>
@@ -2270,7 +2280,7 @@
         <v>7.3330000000000002</v>
       </c>
     </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>23</v>
       </c>
@@ -2344,7 +2354,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>24</v>
       </c>
@@ -2418,7 +2428,7 @@
         <v>7.6669999999999998</v>
       </c>
     </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
       <c r="J27" s="4">
         <v>0.75</v>
       </c>
@@ -2467,7 +2477,7 @@
         <v>7.8330000000000002</v>
       </c>
     </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
       <c r="J28" s="4">
         <v>0.76</v>
       </c>
@@ -2516,7 +2526,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
       <c r="J29" s="4">
         <v>0.77</v>
       </c>
@@ -2565,7 +2575,7 @@
         <v>8.1669999999999998</v>
       </c>
     </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
       <c r="J30" s="4">
         <v>0.78</v>
       </c>
@@ -2614,7 +2624,7 @@
         <v>8.3330000000000002</v>
       </c>
     </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
       <c r="J31" s="4">
         <v>0.79</v>
       </c>
@@ -2663,7 +2673,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="32" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:26" x14ac:dyDescent="0.25">
       <c r="J32" s="4">
         <v>0.8</v>
       </c>
@@ -2712,7 +2722,7 @@
         <v>8.6669999999999998</v>
       </c>
     </row>
-    <row r="33" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="33" spans="10:26" x14ac:dyDescent="0.25">
       <c r="J33" s="4">
         <v>0.81</v>
       </c>
@@ -2761,7 +2771,7 @@
         <v>8.8330000000000002</v>
       </c>
     </row>
-    <row r="34" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="34" spans="10:26" x14ac:dyDescent="0.25">
       <c r="J34" s="4">
         <v>0.82</v>
       </c>
@@ -2810,7 +2820,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="35" spans="10:26" x14ac:dyDescent="0.25">
       <c r="J35" s="4">
         <v>0.83</v>
       </c>
@@ -2859,7 +2869,7 @@
         <v>9.1669999999999998</v>
       </c>
     </row>
-    <row r="36" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="36" spans="10:26" x14ac:dyDescent="0.25">
       <c r="J36" s="4">
         <v>0.84</v>
       </c>
@@ -2908,7 +2918,7 @@
         <v>9.3330000000000002</v>
       </c>
     </row>
-    <row r="37" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="37" spans="10:26" x14ac:dyDescent="0.25">
       <c r="J37" s="4">
         <v>0.85</v>
       </c>
@@ -2957,7 +2967,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="38" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="38" spans="10:26" x14ac:dyDescent="0.25">
       <c r="J38" s="4">
         <v>0.86</v>
       </c>
@@ -3006,7 +3016,7 @@
         <v>9.6669999999999998</v>
       </c>
     </row>
-    <row r="39" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="39" spans="10:26" x14ac:dyDescent="0.25">
       <c r="J39" s="4">
         <v>0.87</v>
       </c>
@@ -3055,7 +3065,7 @@
         <v>9.8330000000000002</v>
       </c>
     </row>
-    <row r="40" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="40" spans="10:26" x14ac:dyDescent="0.25">
       <c r="J40" s="4">
         <v>0.88</v>
       </c>
@@ -3104,7 +3114,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="41" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="41" spans="10:26" x14ac:dyDescent="0.25">
       <c r="J41" s="4">
         <v>0.89</v>
       </c>
@@ -3153,7 +3163,7 @@
         <v>10.125</v>
       </c>
     </row>
-    <row r="42" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="42" spans="10:26" x14ac:dyDescent="0.25">
       <c r="J42" s="4">
         <v>0.9</v>
       </c>
@@ -3202,7 +3212,7 @@
         <v>10.25</v>
       </c>
     </row>
-    <row r="43" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="43" spans="10:26" x14ac:dyDescent="0.25">
       <c r="J43" s="4">
         <v>0.91</v>
       </c>
@@ -3251,7 +3261,7 @@
         <v>10.375</v>
       </c>
     </row>
-    <row r="44" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="44" spans="10:26" x14ac:dyDescent="0.25">
       <c r="J44" s="4">
         <v>0.92</v>
       </c>
@@ -3300,7 +3310,7 @@
         <v>10.5</v>
       </c>
     </row>
-    <row r="45" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="45" spans="10:26" x14ac:dyDescent="0.25">
       <c r="J45" s="4">
         <v>0.93</v>
       </c>
@@ -3349,7 +3359,7 @@
         <v>10.625</v>
       </c>
     </row>
-    <row r="46" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="46" spans="10:26" x14ac:dyDescent="0.25">
       <c r="J46" s="4">
         <v>0.94</v>
       </c>
@@ -3398,7 +3408,7 @@
         <v>10.75</v>
       </c>
     </row>
-    <row r="47" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="47" spans="10:26" x14ac:dyDescent="0.25">
       <c r="J47" s="4">
         <v>0.95</v>
       </c>
@@ -3447,7 +3457,7 @@
         <v>10.875</v>
       </c>
     </row>
-    <row r="48" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="48" spans="10:26" x14ac:dyDescent="0.25">
       <c r="J48" s="4">
         <v>0.96</v>
       </c>
@@ -3496,7 +3506,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="49" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="49" spans="10:26" x14ac:dyDescent="0.25">
       <c r="J49" s="4">
         <v>0.97</v>
       </c>
@@ -3545,7 +3555,7 @@
         <v>11.125</v>
       </c>
     </row>
-    <row r="50" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="50" spans="10:26" x14ac:dyDescent="0.25">
       <c r="J50" s="4">
         <v>0.98</v>
       </c>
@@ -3594,7 +3604,7 @@
         <v>11.25</v>
       </c>
     </row>
-    <row r="51" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="51" spans="10:26" x14ac:dyDescent="0.25">
       <c r="J51" s="4">
         <v>0.99</v>
       </c>
@@ -3643,7 +3653,7 @@
         <v>11.375</v>
       </c>
     </row>
-    <row r="52" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="52" spans="10:26" x14ac:dyDescent="0.25">
       <c r="J52" s="4">
         <v>1</v>
       </c>
@@ -3692,7 +3702,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="53" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="53" spans="10:26" x14ac:dyDescent="0.25">
       <c r="P53" s="4">
         <v>51</v>
       </c>
@@ -3724,7 +3734,7 @@
         <v>11.625</v>
       </c>
     </row>
-    <row r="54" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="54" spans="10:26" x14ac:dyDescent="0.25">
       <c r="P54" s="4">
         <v>52</v>
       </c>
@@ -3756,7 +3766,7 @@
         <v>11.75</v>
       </c>
     </row>
-    <row r="55" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="55" spans="10:26" x14ac:dyDescent="0.25">
       <c r="P55" s="4">
         <v>53</v>
       </c>
@@ -3788,7 +3798,7 @@
         <v>11.875</v>
       </c>
     </row>
-    <row r="56" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="56" spans="10:26" x14ac:dyDescent="0.25">
       <c r="P56" s="4">
         <v>54</v>
       </c>
@@ -3820,7 +3830,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="57" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="57" spans="10:26" x14ac:dyDescent="0.25">
       <c r="P57" s="4">
         <v>55</v>
       </c>
@@ -3852,7 +3862,7 @@
         <v>12.111000000000001</v>
       </c>
     </row>
-    <row r="58" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="58" spans="10:26" x14ac:dyDescent="0.25">
       <c r="P58" s="4">
         <v>56</v>
       </c>
@@ -3884,7 +3894,7 @@
         <v>12.222</v>
       </c>
     </row>
-    <row r="59" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="59" spans="10:26" x14ac:dyDescent="0.25">
       <c r="P59" s="4">
         <v>57</v>
       </c>
@@ -3916,7 +3926,7 @@
         <v>12.333</v>
       </c>
     </row>
-    <row r="60" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="60" spans="10:26" x14ac:dyDescent="0.25">
       <c r="P60" s="4">
         <v>58</v>
       </c>
@@ -3948,7 +3958,7 @@
         <v>12.444000000000001</v>
       </c>
     </row>
-    <row r="61" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="61" spans="10:26" x14ac:dyDescent="0.25">
       <c r="P61" s="4">
         <v>59</v>
       </c>
@@ -3980,7 +3990,7 @@
         <v>12.555999999999999</v>
       </c>
     </row>
-    <row r="62" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="62" spans="10:26" x14ac:dyDescent="0.25">
       <c r="P62" s="4">
         <v>60</v>
       </c>
@@ -4012,7 +4022,7 @@
         <v>12.667</v>
       </c>
     </row>
-    <row r="63" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="63" spans="10:26" x14ac:dyDescent="0.25">
       <c r="P63" s="4">
         <v>61</v>
       </c>
@@ -4044,7 +4054,7 @@
         <v>12.778</v>
       </c>
     </row>
-    <row r="64" spans="10:26" x14ac:dyDescent="0.3">
+    <row r="64" spans="10:26" x14ac:dyDescent="0.25">
       <c r="P64" s="4">
         <v>62</v>
       </c>
@@ -4076,7 +4086,7 @@
         <v>12.888999999999999</v>
       </c>
     </row>
-    <row r="65" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="65" spans="16:26" x14ac:dyDescent="0.25">
       <c r="P65" s="4">
         <v>63</v>
       </c>
@@ -4108,7 +4118,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="66" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="66" spans="16:26" x14ac:dyDescent="0.25">
       <c r="P66" s="4">
         <v>64</v>
       </c>
@@ -4140,7 +4150,7 @@
         <v>13.111000000000001</v>
       </c>
     </row>
-    <row r="67" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="67" spans="16:26" x14ac:dyDescent="0.25">
       <c r="P67" s="4">
         <v>65</v>
       </c>
@@ -4172,7 +4182,7 @@
         <v>13.222</v>
       </c>
     </row>
-    <row r="68" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="68" spans="16:26" x14ac:dyDescent="0.25">
       <c r="P68" s="4">
         <v>66</v>
       </c>
@@ -4204,7 +4214,7 @@
         <v>13.333</v>
       </c>
     </row>
-    <row r="69" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="69" spans="16:26" x14ac:dyDescent="0.25">
       <c r="P69" s="4">
         <v>67</v>
       </c>
@@ -4236,7 +4246,7 @@
         <v>13.444000000000001</v>
       </c>
     </row>
-    <row r="70" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="70" spans="16:26" x14ac:dyDescent="0.25">
       <c r="P70" s="4">
         <v>68</v>
       </c>
@@ -4268,7 +4278,7 @@
         <v>13.555999999999999</v>
       </c>
     </row>
-    <row r="71" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="71" spans="16:26" x14ac:dyDescent="0.25">
       <c r="P71" s="4">
         <v>69</v>
       </c>
@@ -4300,7 +4310,7 @@
         <v>13.667</v>
       </c>
     </row>
-    <row r="72" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="72" spans="16:26" x14ac:dyDescent="0.25">
       <c r="P72" s="4">
         <v>70</v>
       </c>
@@ -4332,7 +4342,7 @@
         <v>13.778</v>
       </c>
     </row>
-    <row r="73" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="73" spans="16:26" x14ac:dyDescent="0.25">
       <c r="P73" s="4">
         <v>71</v>
       </c>
@@ -4364,7 +4374,7 @@
         <v>13.888999999999999</v>
       </c>
     </row>
-    <row r="74" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="74" spans="16:26" x14ac:dyDescent="0.25">
       <c r="P74" s="4">
         <v>72</v>
       </c>
@@ -4396,7 +4406,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="75" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="75" spans="16:26" x14ac:dyDescent="0.25">
       <c r="P75" s="4">
         <v>73</v>
       </c>
@@ -4428,7 +4438,7 @@
         <v>14.1</v>
       </c>
     </row>
-    <row r="76" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="76" spans="16:26" x14ac:dyDescent="0.25">
       <c r="P76" s="4">
         <v>74</v>
       </c>
@@ -4460,7 +4470,7 @@
         <v>14.2</v>
       </c>
     </row>
-    <row r="77" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="77" spans="16:26" x14ac:dyDescent="0.25">
       <c r="P77" s="4">
         <v>75</v>
       </c>
@@ -4492,7 +4502,7 @@
         <v>14.3</v>
       </c>
     </row>
-    <row r="78" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="78" spans="16:26" x14ac:dyDescent="0.25">
       <c r="P78" s="4">
         <v>76</v>
       </c>
@@ -4524,7 +4534,7 @@
         <v>14.4</v>
       </c>
     </row>
-    <row r="79" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="79" spans="16:26" x14ac:dyDescent="0.25">
       <c r="P79" s="4">
         <v>77</v>
       </c>
@@ -4556,7 +4566,7 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="80" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="80" spans="16:26" x14ac:dyDescent="0.25">
       <c r="P80" s="4">
         <v>78</v>
       </c>
@@ -4588,7 +4598,7 @@
         <v>14.6</v>
       </c>
     </row>
-    <row r="81" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="81" spans="16:26" x14ac:dyDescent="0.25">
       <c r="P81" s="4">
         <v>79</v>
       </c>
@@ -4620,7 +4630,7 @@
         <v>14.7</v>
       </c>
     </row>
-    <row r="82" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="82" spans="16:26" x14ac:dyDescent="0.25">
       <c r="P82" s="4">
         <v>80</v>
       </c>
@@ -4652,7 +4662,7 @@
         <v>14.8</v>
       </c>
     </row>
-    <row r="83" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="83" spans="16:26" x14ac:dyDescent="0.25">
       <c r="P83" s="4">
         <v>81</v>
       </c>
@@ -4684,7 +4694,7 @@
         <v>14.9</v>
       </c>
     </row>
-    <row r="84" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="84" spans="16:26" x14ac:dyDescent="0.25">
       <c r="P84" s="4">
         <v>82</v>
       </c>
@@ -4716,7 +4726,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="85" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="85" spans="16:26" x14ac:dyDescent="0.25">
       <c r="P85" s="4">
         <v>83</v>
       </c>
@@ -4748,7 +4758,7 @@
         <v>15.090999999999999</v>
       </c>
     </row>
-    <row r="86" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="86" spans="16:26" x14ac:dyDescent="0.25">
       <c r="P86" s="4">
         <v>84</v>
       </c>
@@ -4780,7 +4790,7 @@
         <v>15.182</v>
       </c>
     </row>
-    <row r="87" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="87" spans="16:26" x14ac:dyDescent="0.25">
       <c r="P87" s="4">
         <v>150</v>
       </c>
@@ -4812,7 +4822,7 @@
         <v>15.273</v>
       </c>
     </row>
-    <row r="88" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="88" spans="16:26" x14ac:dyDescent="0.25">
       <c r="V88" s="4">
         <v>86</v>
       </c>
@@ -4829,7 +4839,7 @@
         <v>15.364000000000001</v>
       </c>
     </row>
-    <row r="89" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="89" spans="16:26" x14ac:dyDescent="0.25">
       <c r="V89" s="4">
         <v>87</v>
       </c>
@@ -4846,7 +4856,7 @@
         <v>15.455</v>
       </c>
     </row>
-    <row r="90" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="90" spans="16:26" x14ac:dyDescent="0.25">
       <c r="V90" s="4">
         <v>88</v>
       </c>
@@ -4863,7 +4873,7 @@
         <v>15.545</v>
       </c>
     </row>
-    <row r="91" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="91" spans="16:26" x14ac:dyDescent="0.25">
       <c r="V91" s="4">
         <v>89</v>
       </c>
@@ -4880,7 +4890,7 @@
         <v>15.635999999999999</v>
       </c>
     </row>
-    <row r="92" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="92" spans="16:26" x14ac:dyDescent="0.25">
       <c r="V92" s="4">
         <v>90</v>
       </c>
@@ -4897,7 +4907,7 @@
         <v>15.727</v>
       </c>
     </row>
-    <row r="93" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="93" spans="16:26" x14ac:dyDescent="0.25">
       <c r="V93" s="4">
         <v>91</v>
       </c>
@@ -4914,7 +4924,7 @@
         <v>15.818</v>
       </c>
     </row>
-    <row r="94" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="94" spans="16:26" x14ac:dyDescent="0.25">
       <c r="V94" s="4">
         <v>92</v>
       </c>
@@ -4931,7 +4941,7 @@
         <v>15.909000000000001</v>
       </c>
     </row>
-    <row r="95" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="95" spans="16:26" x14ac:dyDescent="0.25">
       <c r="V95" s="4">
         <v>93</v>
       </c>
@@ -4948,7 +4958,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="96" spans="16:26" x14ac:dyDescent="0.3">
+    <row r="96" spans="16:26" x14ac:dyDescent="0.25">
       <c r="V96" s="4">
         <v>94</v>
       </c>
@@ -4965,7 +4975,7 @@
         <v>16.091000000000001</v>
       </c>
     </row>
-    <row r="97" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="97" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V97" s="4">
         <v>95</v>
       </c>
@@ -4982,7 +4992,7 @@
         <v>16.181999999999999</v>
       </c>
     </row>
-    <row r="98" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="98" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V98" s="4">
         <v>96</v>
       </c>
@@ -4999,7 +5009,7 @@
         <v>16.273</v>
       </c>
     </row>
-    <row r="99" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="99" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V99" s="4">
         <v>97</v>
       </c>
@@ -5016,7 +5026,7 @@
         <v>16.364000000000001</v>
       </c>
     </row>
-    <row r="100" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="100" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V100" s="4">
         <v>98</v>
       </c>
@@ -5033,7 +5043,7 @@
         <v>16.454999999999998</v>
       </c>
     </row>
-    <row r="101" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="101" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V101" s="4">
         <v>99</v>
       </c>
@@ -5050,7 +5060,7 @@
         <v>16.545000000000002</v>
       </c>
     </row>
-    <row r="102" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="102" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V102" s="4">
         <v>100</v>
       </c>
@@ -5067,7 +5077,7 @@
         <v>16.635999999999999</v>
       </c>
     </row>
-    <row r="103" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="103" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V103" s="4">
         <v>101</v>
       </c>
@@ -5084,7 +5094,7 @@
         <v>16.727</v>
       </c>
     </row>
-    <row r="104" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="104" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V104" s="4">
         <v>102</v>
       </c>
@@ -5101,7 +5111,7 @@
         <v>16.818000000000001</v>
       </c>
     </row>
-    <row r="105" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="105" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V105" s="4">
         <v>103</v>
       </c>
@@ -5118,7 +5128,7 @@
         <v>16.908999999999999</v>
       </c>
     </row>
-    <row r="106" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="106" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V106" s="4">
         <v>104</v>
       </c>
@@ -5135,7 +5145,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="107" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="107" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V107" s="4">
         <v>105</v>
       </c>
@@ -5152,7 +5162,7 @@
         <v>17.082999999999998</v>
       </c>
     </row>
-    <row r="108" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="108" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V108" s="4">
         <v>106</v>
       </c>
@@ -5169,7 +5179,7 @@
         <v>17.167000000000002</v>
       </c>
     </row>
-    <row r="109" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="109" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V109" s="4">
         <v>107</v>
       </c>
@@ -5186,7 +5196,7 @@
         <v>17.25</v>
       </c>
     </row>
-    <row r="110" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="110" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V110" s="4">
         <v>108</v>
       </c>
@@ -5203,7 +5213,7 @@
         <v>17.332999999999998</v>
       </c>
     </row>
-    <row r="111" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="111" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V111" s="4">
         <v>109</v>
       </c>
@@ -5220,7 +5230,7 @@
         <v>17.417000000000002</v>
       </c>
     </row>
-    <row r="112" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="112" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V112" s="4">
         <v>110</v>
       </c>
@@ -5237,7 +5247,7 @@
         <v>17.5</v>
       </c>
     </row>
-    <row r="113" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="113" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V113" s="4">
         <v>111</v>
       </c>
@@ -5254,7 +5264,7 @@
         <v>17.582999999999998</v>
       </c>
     </row>
-    <row r="114" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="114" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V114" s="4">
         <v>112</v>
       </c>
@@ -5271,7 +5281,7 @@
         <v>17.667000000000002</v>
       </c>
     </row>
-    <row r="115" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="115" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V115" s="4">
         <v>113</v>
       </c>
@@ -5288,7 +5298,7 @@
         <v>17.75</v>
       </c>
     </row>
-    <row r="116" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="116" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V116" s="4">
         <v>114</v>
       </c>
@@ -5305,7 +5315,7 @@
         <v>17.832999999999998</v>
       </c>
     </row>
-    <row r="117" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="117" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V117" s="4">
         <v>115</v>
       </c>
@@ -5322,7 +5332,7 @@
         <v>17.917000000000002</v>
       </c>
     </row>
-    <row r="118" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="118" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V118" s="4">
         <v>116</v>
       </c>
@@ -5339,7 +5349,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="119" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="119" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V119" s="4">
         <v>117</v>
       </c>
@@ -5356,7 +5366,7 @@
         <v>18.082999999999998</v>
       </c>
     </row>
-    <row r="120" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="120" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V120" s="4">
         <v>118</v>
       </c>
@@ -5373,7 +5383,7 @@
         <v>18.167000000000002</v>
       </c>
     </row>
-    <row r="121" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="121" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V121" s="4">
         <v>119</v>
       </c>
@@ -5390,7 +5400,7 @@
         <v>18.25</v>
       </c>
     </row>
-    <row r="122" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="122" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V122" s="4">
         <v>120</v>
       </c>
@@ -5407,7 +5417,7 @@
         <v>18.332999999999998</v>
       </c>
     </row>
-    <row r="123" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="123" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V123" s="4">
         <v>121</v>
       </c>
@@ -5424,7 +5434,7 @@
         <v>18.417000000000002</v>
       </c>
     </row>
-    <row r="124" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="124" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V124" s="4">
         <v>122</v>
       </c>
@@ -5441,7 +5451,7 @@
         <v>18.5</v>
       </c>
     </row>
-    <row r="125" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="125" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V125" s="4">
         <v>123</v>
       </c>
@@ -5458,7 +5468,7 @@
         <v>18.582999999999998</v>
       </c>
     </row>
-    <row r="126" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="126" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V126" s="4">
         <v>124</v>
       </c>
@@ -5475,7 +5485,7 @@
         <v>18.667000000000002</v>
       </c>
     </row>
-    <row r="127" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="127" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V127" s="4">
         <v>125</v>
       </c>
@@ -5492,7 +5502,7 @@
         <v>18.75</v>
       </c>
     </row>
-    <row r="128" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="128" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V128" s="4">
         <v>126</v>
       </c>
@@ -5509,7 +5519,7 @@
         <v>18.832999999999998</v>
       </c>
     </row>
-    <row r="129" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="129" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V129" s="4">
         <v>127</v>
       </c>
@@ -5526,7 +5536,7 @@
         <v>18.917000000000002</v>
       </c>
     </row>
-    <row r="130" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="130" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V130" s="4">
         <v>128</v>
       </c>
@@ -5543,7 +5553,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="131" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="131" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V131" s="4">
         <v>129</v>
       </c>
@@ -5560,7 +5570,7 @@
         <v>19.077000000000002</v>
       </c>
     </row>
-    <row r="132" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="132" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V132" s="4">
         <v>130</v>
       </c>
@@ -5577,7 +5587,7 @@
         <v>19.154</v>
       </c>
     </row>
-    <row r="133" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="133" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V133" s="4">
         <v>131</v>
       </c>
@@ -5594,7 +5604,7 @@
         <v>19.231000000000002</v>
       </c>
     </row>
-    <row r="134" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="134" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V134" s="4">
         <v>132</v>
       </c>
@@ -5611,7 +5621,7 @@
         <v>19.308</v>
       </c>
     </row>
-    <row r="135" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="135" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V135" s="4">
         <v>133</v>
       </c>
@@ -5628,7 +5638,7 @@
         <v>19.385000000000002</v>
       </c>
     </row>
-    <row r="136" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="136" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V136" s="4">
         <v>134</v>
       </c>
@@ -5645,7 +5655,7 @@
         <v>19.462</v>
       </c>
     </row>
-    <row r="137" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="137" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V137" s="4">
         <v>135</v>
       </c>
@@ -5662,7 +5672,7 @@
         <v>19.538</v>
       </c>
     </row>
-    <row r="138" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="138" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V138" s="4">
         <v>136</v>
       </c>
@@ -5679,7 +5689,7 @@
         <v>19.614999999999998</v>
       </c>
     </row>
-    <row r="139" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="139" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V139" s="4">
         <v>137</v>
       </c>
@@ -5696,7 +5706,7 @@
         <v>19.692</v>
       </c>
     </row>
-    <row r="140" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="140" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V140" s="4">
         <v>138</v>
       </c>
@@ -5713,7 +5723,7 @@
         <v>19.768999999999998</v>
       </c>
     </row>
-    <row r="141" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="141" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V141" s="4">
         <v>139</v>
       </c>
@@ -5730,7 +5740,7 @@
         <v>19.846</v>
       </c>
     </row>
-    <row r="142" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="142" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V142" s="4">
         <v>140</v>
       </c>
@@ -5747,7 +5757,7 @@
         <v>19.922999999999998</v>
       </c>
     </row>
-    <row r="143" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="143" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V143" s="4">
         <v>141</v>
       </c>
@@ -5764,7 +5774,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="144" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="144" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V144" s="4">
         <v>142</v>
       </c>
@@ -5781,7 +5791,7 @@
         <v>20.077000000000002</v>
       </c>
     </row>
-    <row r="145" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="145" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V145" s="4">
         <v>143</v>
       </c>
@@ -5798,7 +5808,7 @@
         <v>20.154</v>
       </c>
     </row>
-    <row r="146" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="146" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V146" s="4">
         <v>144</v>
       </c>
@@ -5815,7 +5825,7 @@
         <v>20.231000000000002</v>
       </c>
     </row>
-    <row r="147" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="147" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V147" s="4">
         <v>145</v>
       </c>
@@ -5832,7 +5842,7 @@
         <v>20.268000000000001</v>
       </c>
     </row>
-    <row r="148" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="148" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V148" s="4">
         <v>146</v>
       </c>
@@ -5849,7 +5859,7 @@
         <v>20.268000000000001</v>
       </c>
     </row>
-    <row r="149" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="149" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V149" s="4">
         <v>147</v>
       </c>
@@ -5866,7 +5876,7 @@
         <v>20.268000000000001</v>
       </c>
     </row>
-    <row r="150" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="150" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V150" s="4">
         <v>148</v>
       </c>
@@ -5883,7 +5893,7 @@
         <v>20.268000000000001</v>
       </c>
     </row>
-    <row r="151" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="151" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V151" s="4">
         <v>149</v>
       </c>
@@ -5900,7 +5910,7 @@
         <v>20.268000000000001</v>
       </c>
     </row>
-    <row r="152" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="152" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V152" s="4">
         <v>150</v>
       </c>
@@ -5917,7 +5927,7 @@
         <v>20.268000000000001</v>
       </c>
     </row>
-    <row r="153" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="153" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V153" s="4">
         <v>151</v>
       </c>
@@ -5934,7 +5944,7 @@
         <v>20.268000000000001</v>
       </c>
     </row>
-    <row r="154" spans="22:26" x14ac:dyDescent="0.3">
+    <row r="154" spans="22:26" x14ac:dyDescent="0.25">
       <c r="V154" s="4">
         <v>152</v>
       </c>
@@ -5955,4 +5965,1141 @@
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C8D9161-C241-47C4-989B-A93783CCB88D}">
+  <dimension ref="A1:H138"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="4">
+        <v>0</v>
+      </c>
+      <c r="B2" s="4">
+        <v>98</v>
+      </c>
+      <c r="C2" s="4">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="B3" s="4">
+        <v>95.751999999999995</v>
+      </c>
+      <c r="C3" s="4">
+        <v>55.725000000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="4">
+        <v>0.02</v>
+      </c>
+      <c r="B4" s="4">
+        <v>94.221999999999994</v>
+      </c>
+      <c r="C4" s="4">
+        <v>54.771999999999998</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="4">
+        <v>0.03</v>
+      </c>
+      <c r="B5" s="4">
+        <v>93.073999999999998</v>
+      </c>
+      <c r="C5" s="4">
+        <v>54.127000000000002</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="4">
+        <v>0.04</v>
+      </c>
+      <c r="B6" s="4">
+        <v>92.242000000000004</v>
+      </c>
+      <c r="C6" s="4">
+        <v>53.642000000000003</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="4">
+        <v>0.05</v>
+      </c>
+      <c r="B7" s="4">
+        <v>91.49</v>
+      </c>
+      <c r="C7" s="4">
+        <v>53.22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="4">
+        <v>0.06</v>
+      </c>
+      <c r="B8" s="4">
+        <v>90.85</v>
+      </c>
+      <c r="C8" s="4">
+        <v>52.875999999999998</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="4">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="B9" s="4">
+        <v>90.370999999999995</v>
+      </c>
+      <c r="C9" s="4">
+        <v>52.606000000000002</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="4">
+        <v>0.08</v>
+      </c>
+      <c r="B10" s="4">
+        <v>89.914000000000001</v>
+      </c>
+      <c r="C10" s="4">
+        <v>52.348999999999997</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="4">
+        <v>0.09</v>
+      </c>
+      <c r="B11" s="4">
+        <v>89.478999999999999</v>
+      </c>
+      <c r="C11" s="4">
+        <v>52.104999999999997</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="B12" s="4">
+        <v>89.063999999999993</v>
+      </c>
+      <c r="C12" s="4">
+        <v>51.872</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="4">
+        <v>0.11</v>
+      </c>
+      <c r="B13" s="4">
+        <v>88.668000000000006</v>
+      </c>
+      <c r="C13" s="4">
+        <v>51.649000000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="4">
+        <v>0.12</v>
+      </c>
+      <c r="B14" s="4">
+        <v>88.289000000000001</v>
+      </c>
+      <c r="C14" s="4">
+        <v>51.436</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="4">
+        <v>0.13</v>
+      </c>
+      <c r="B15" s="4">
+        <v>87.938999999999993</v>
+      </c>
+      <c r="C15" s="4">
+        <v>51.232999999999997</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="4">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="B16" s="4">
+        <v>87.65</v>
+      </c>
+      <c r="C16" s="4">
+        <v>51.037999999999997</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="4">
+        <v>0.15</v>
+      </c>
+      <c r="B17" s="4">
+        <v>87.37</v>
+      </c>
+      <c r="C17" s="4">
+        <v>50.875</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="4">
+        <v>0.16</v>
+      </c>
+      <c r="B18" s="4">
+        <v>87.097999999999999</v>
+      </c>
+      <c r="C18" s="4">
+        <v>50.722999999999999</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="4">
+        <v>0.17</v>
+      </c>
+      <c r="B19" s="4">
+        <v>86.834999999999994</v>
+      </c>
+      <c r="C19" s="4">
+        <v>50.576000000000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="4">
+        <v>0.18</v>
+      </c>
+      <c r="B20" s="4">
+        <v>86.578999999999994</v>
+      </c>
+      <c r="C20" s="4">
+        <v>50.433999999999997</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="4">
+        <v>0.19</v>
+      </c>
+      <c r="B21" s="4">
+        <v>86.331000000000003</v>
+      </c>
+      <c r="C21" s="4">
+        <v>50.295000000000002</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="4">
+        <v>0.2</v>
+      </c>
+      <c r="B22" s="4">
+        <v>86.088999999999999</v>
+      </c>
+      <c r="C22" s="4">
+        <v>50.161000000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="4">
+        <v>0.21</v>
+      </c>
+      <c r="B23" s="4">
+        <v>85.864000000000004</v>
+      </c>
+      <c r="C23" s="4">
+        <v>50.03</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="4">
+        <v>0.22</v>
+      </c>
+      <c r="B24" s="4">
+        <v>85.65</v>
+      </c>
+      <c r="C24" s="4">
+        <v>49.908999999999999</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="4">
+        <v>0.23</v>
+      </c>
+      <c r="B25" s="4">
+        <v>85.441999999999993</v>
+      </c>
+      <c r="C25" s="4">
+        <v>49.792999999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="4">
+        <v>0.24</v>
+      </c>
+      <c r="B26" s="4">
+        <v>85.238</v>
+      </c>
+      <c r="C26" s="4">
+        <v>49.679000000000002</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="4">
+        <v>0.25</v>
+      </c>
+      <c r="B27" s="4">
+        <v>85.039000000000001</v>
+      </c>
+      <c r="C27" s="4">
+        <v>49.569000000000003</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="4">
+        <v>0.26</v>
+      </c>
+      <c r="B28" s="4">
+        <v>84.844999999999999</v>
+      </c>
+      <c r="C28" s="4">
+        <v>49.46</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="4">
+        <v>0.27</v>
+      </c>
+      <c r="B29" s="4">
+        <v>84.655000000000001</v>
+      </c>
+      <c r="C29" s="4">
+        <v>49.354999999999997</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="4">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="B30" s="4">
+        <v>84.47</v>
+      </c>
+      <c r="C30" s="4">
+        <v>49.252000000000002</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="4">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="B31" s="4">
+        <v>84.287999999999997</v>
+      </c>
+      <c r="C31" s="4">
+        <v>49.151000000000003</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="4">
+        <v>0.3</v>
+      </c>
+      <c r="B32" s="4">
+        <v>84.111000000000004</v>
+      </c>
+      <c r="C32" s="4">
+        <v>49.052</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="4">
+        <v>0.31</v>
+      </c>
+      <c r="B33" s="4">
+        <v>83.941000000000003</v>
+      </c>
+      <c r="C33" s="4">
+        <v>48.957000000000001</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="4">
+        <v>0.32</v>
+      </c>
+      <c r="B34" s="4">
+        <v>83.778999999999996</v>
+      </c>
+      <c r="C34" s="4">
+        <v>48.866999999999997</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="4">
+        <v>0.33</v>
+      </c>
+      <c r="B35" s="4">
+        <v>83.62</v>
+      </c>
+      <c r="C35" s="4">
+        <v>48.779000000000003</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="4">
+        <v>0.34</v>
+      </c>
+      <c r="B36" s="4">
+        <v>83.465000000000003</v>
+      </c>
+      <c r="C36" s="4">
+        <v>48.692</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="4">
+        <v>0.35</v>
+      </c>
+      <c r="B37" s="4">
+        <v>83.311999999999998</v>
+      </c>
+      <c r="C37" s="4">
+        <v>48.606999999999999</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="4">
+        <v>0.36</v>
+      </c>
+      <c r="B38" s="4">
+        <v>83.162000000000006</v>
+      </c>
+      <c r="C38" s="4">
+        <v>48.524000000000001</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="4">
+        <v>0.37</v>
+      </c>
+      <c r="B39" s="4">
+        <v>83.015000000000001</v>
+      </c>
+      <c r="C39" s="4">
+        <v>48.442</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="4">
+        <v>0.38</v>
+      </c>
+      <c r="B40" s="4">
+        <v>82.876000000000005</v>
+      </c>
+      <c r="C40" s="4">
+        <v>48.362000000000002</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="4">
+        <v>0.39</v>
+      </c>
+      <c r="B41" s="4">
+        <v>82.739000000000004</v>
+      </c>
+      <c r="C41" s="4">
+        <v>48.283000000000001</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="4">
+        <v>0.4</v>
+      </c>
+      <c r="B42" s="4">
+        <v>82.605000000000004</v>
+      </c>
+      <c r="C42" s="4">
+        <v>48.204999999999998</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="4">
+        <v>0.41</v>
+      </c>
+      <c r="B43" s="4">
+        <v>82.472999999999999</v>
+      </c>
+      <c r="C43" s="4">
+        <v>48.128999999999998</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" s="4">
+        <v>0.42</v>
+      </c>
+      <c r="B44" s="4">
+        <v>82.343000000000004</v>
+      </c>
+      <c r="C44" s="4">
+        <v>48.054000000000002</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" s="4">
+        <v>0.43</v>
+      </c>
+      <c r="B45" s="4">
+        <v>82.215000000000003</v>
+      </c>
+      <c r="C45" s="4">
+        <v>47.981000000000002</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" s="4">
+        <v>0.44</v>
+      </c>
+      <c r="B46" s="4">
+        <v>82.088999999999999</v>
+      </c>
+      <c r="C46" s="4">
+        <v>47.911000000000001</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" s="4">
+        <v>0.45</v>
+      </c>
+      <c r="B47" s="4">
+        <v>81.963999999999999</v>
+      </c>
+      <c r="C47" s="4">
+        <v>47.843000000000004</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" s="4">
+        <v>0.46</v>
+      </c>
+      <c r="B48" s="4">
+        <v>81.841999999999999</v>
+      </c>
+      <c r="C48" s="4">
+        <v>47.774999999999999</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" s="4">
+        <v>0.47</v>
+      </c>
+      <c r="B49" s="4">
+        <v>81.721999999999994</v>
+      </c>
+      <c r="C49" s="4">
+        <v>47.707999999999998</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="4">
+        <v>0.48</v>
+      </c>
+      <c r="B50" s="4">
+        <v>81.602999999999994</v>
+      </c>
+      <c r="C50" s="4">
+        <v>47.643000000000001</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="4">
+        <v>0.49</v>
+      </c>
+      <c r="B51" s="4">
+        <v>81.486000000000004</v>
+      </c>
+      <c r="C51" s="4">
+        <v>47.578000000000003</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="B52" s="4">
+        <v>81.370999999999995</v>
+      </c>
+      <c r="C52" s="4">
+        <v>47.514000000000003</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="4">
+        <v>0.51</v>
+      </c>
+      <c r="B53" s="4">
+        <v>81.257999999999996</v>
+      </c>
+      <c r="C53" s="4">
+        <v>47.451999999999998</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="4">
+        <v>0.52</v>
+      </c>
+      <c r="B54" s="4">
+        <v>81.146000000000001</v>
+      </c>
+      <c r="C54" s="4">
+        <v>47.39</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="4">
+        <v>0.53</v>
+      </c>
+      <c r="B55" s="4">
+        <v>81.036000000000001</v>
+      </c>
+      <c r="C55" s="4">
+        <v>47.329000000000001</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" s="4">
+        <v>0.54</v>
+      </c>
+      <c r="B56" s="4">
+        <v>80.930000000000007</v>
+      </c>
+      <c r="C56" s="4">
+        <v>47.268999999999998</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="4">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="B57" s="4">
+        <v>80.825000000000003</v>
+      </c>
+      <c r="C57" s="4">
+        <v>47.209000000000003</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" s="4">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="B58" s="4">
+        <v>80.721999999999994</v>
+      </c>
+      <c r="C58" s="4">
+        <v>47.151000000000003</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" s="4">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="B59" s="4">
+        <v>80.62</v>
+      </c>
+      <c r="C59" s="4">
+        <v>47.093000000000004</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" s="4">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="B60" s="4">
+        <v>80.52</v>
+      </c>
+      <c r="C60" s="4">
+        <v>47.036999999999999</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" s="4">
+        <v>0.59</v>
+      </c>
+      <c r="B61" s="4">
+        <v>80.421000000000006</v>
+      </c>
+      <c r="C61" s="4">
+        <v>46.981000000000002</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" s="4">
+        <v>0.6</v>
+      </c>
+      <c r="B62" s="4">
+        <v>80.322999999999993</v>
+      </c>
+      <c r="C62" s="4">
+        <v>46.927</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" s="4">
+        <v>0.61</v>
+      </c>
+      <c r="B63" s="4">
+        <v>80.225999999999999</v>
+      </c>
+      <c r="C63" s="4">
+        <v>46.874000000000002</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" s="4">
+        <v>0.62</v>
+      </c>
+      <c r="B64" s="4">
+        <v>80.131</v>
+      </c>
+      <c r="C64" s="4">
+        <v>46.820999999999998</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" s="4">
+        <v>0.63</v>
+      </c>
+      <c r="B65" s="4">
+        <v>80.036000000000001</v>
+      </c>
+      <c r="C65" s="4">
+        <v>46.768999999999998</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" s="4">
+        <v>0.64</v>
+      </c>
+      <c r="B66" s="4">
+        <v>79.942999999999998</v>
+      </c>
+      <c r="C66" s="4">
+        <v>46.716999999999999</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67" s="4">
+        <v>0.65</v>
+      </c>
+      <c r="B67" s="4">
+        <v>79.850999999999999</v>
+      </c>
+      <c r="C67" s="4">
+        <v>46.667000000000002</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68" s="4">
+        <v>0.66</v>
+      </c>
+      <c r="B68" s="4">
+        <v>79.760000000000005</v>
+      </c>
+      <c r="C68" s="4">
+        <v>46.616</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69" s="4">
+        <v>0.67</v>
+      </c>
+      <c r="B69" s="4">
+        <v>79.67</v>
+      </c>
+      <c r="C69" s="4">
+        <v>46.567</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70" s="4">
+        <v>0.68</v>
+      </c>
+      <c r="B70" s="4">
+        <v>79.581000000000003</v>
+      </c>
+      <c r="C70" s="4">
+        <v>46.518000000000001</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71" s="4">
+        <v>0.69</v>
+      </c>
+      <c r="B71" s="4">
+        <v>79.494</v>
+      </c>
+      <c r="C71" s="4">
+        <v>46.469000000000001</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72" s="4">
+        <v>0.7</v>
+      </c>
+      <c r="B72" s="4">
+        <v>79.406999999999996</v>
+      </c>
+      <c r="C72" s="4">
+        <v>46.421999999999997</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73" s="4">
+        <v>0.71</v>
+      </c>
+      <c r="B73" s="4">
+        <v>79.320999999999998</v>
+      </c>
+      <c r="C73" s="4">
+        <v>46.374000000000002</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74" s="4">
+        <v>0.72</v>
+      </c>
+      <c r="B74" s="4">
+        <v>79.236000000000004</v>
+      </c>
+      <c r="C74" s="4">
+        <v>46.328000000000003</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A75" s="4">
+        <v>0.73</v>
+      </c>
+      <c r="B75" s="4">
+        <v>79.153000000000006</v>
+      </c>
+      <c r="C75" s="4">
+        <v>46.280999999999999</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A76" s="4">
+        <v>0.74</v>
+      </c>
+      <c r="B76" s="4">
+        <v>79.069999999999993</v>
+      </c>
+      <c r="C76" s="4">
+        <v>46.235999999999997</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A77" s="4">
+        <v>0.75</v>
+      </c>
+      <c r="B77" s="4">
+        <v>78.988</v>
+      </c>
+      <c r="C77" s="4">
+        <v>46.19</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A78" s="4">
+        <v>0.76</v>
+      </c>
+      <c r="B78" s="4">
+        <v>78.908000000000001</v>
+      </c>
+      <c r="C78" s="4">
+        <v>46.146000000000001</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79" s="4">
+        <v>0.77</v>
+      </c>
+      <c r="B79" s="4">
+        <v>78.828999999999994</v>
+      </c>
+      <c r="C79" s="4">
+        <v>46.101999999999997</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A80" s="4">
+        <v>0.78</v>
+      </c>
+      <c r="B80" s="4">
+        <v>78.751000000000005</v>
+      </c>
+      <c r="C80" s="4">
+        <v>46.058</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A81" s="4">
+        <v>0.79</v>
+      </c>
+      <c r="B81" s="4">
+        <v>78.673000000000002</v>
+      </c>
+      <c r="C81" s="4">
+        <v>46.015000000000001</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82" s="4">
+        <v>0.8</v>
+      </c>
+      <c r="B82" s="4">
+        <v>78.596000000000004</v>
+      </c>
+      <c r="C82" s="4">
+        <v>45.972000000000001</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83" s="4">
+        <v>0.81</v>
+      </c>
+      <c r="B83" s="4">
+        <v>78.52</v>
+      </c>
+      <c r="C83" s="4">
+        <v>45.930999999999997</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84" s="4">
+        <v>0.82</v>
+      </c>
+      <c r="B84" s="4">
+        <v>78.444999999999993</v>
+      </c>
+      <c r="C84" s="4">
+        <v>45.889000000000003</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A85" s="4">
+        <v>0.83</v>
+      </c>
+      <c r="B85" s="4">
+        <v>78.370999999999995</v>
+      </c>
+      <c r="C85" s="4">
+        <v>45.847999999999999</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A86" s="4">
+        <v>0.84</v>
+      </c>
+      <c r="B86" s="4">
+        <v>78.296999999999997</v>
+      </c>
+      <c r="C86" s="4">
+        <v>45.808</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A87" s="4">
+        <v>0.85</v>
+      </c>
+      <c r="B87" s="4">
+        <v>78.224000000000004</v>
+      </c>
+      <c r="C87" s="4">
+        <v>45.767000000000003</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A88" s="4">
+        <v>0.86</v>
+      </c>
+      <c r="B88" s="4">
+        <v>78.150999999999996</v>
+      </c>
+      <c r="C88" s="4">
+        <v>45.728000000000002</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A89" s="4">
+        <v>0.87</v>
+      </c>
+      <c r="B89" s="4">
+        <v>78.08</v>
+      </c>
+      <c r="C89" s="4">
+        <v>45.688000000000002</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A90" s="4">
+        <v>0.88</v>
+      </c>
+      <c r="B90" s="4">
+        <v>78.009</v>
+      </c>
+      <c r="C90" s="4">
+        <v>45.649000000000001</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A91" s="4">
+        <v>0.89</v>
+      </c>
+      <c r="B91" s="4">
+        <v>77.938999999999993</v>
+      </c>
+      <c r="C91" s="4">
+        <v>45.61</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A92" s="4">
+        <v>0.9</v>
+      </c>
+      <c r="B92" s="4">
+        <v>77.869</v>
+      </c>
+      <c r="C92" s="4">
+        <v>45.572000000000003</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A93" s="4">
+        <v>0.91</v>
+      </c>
+      <c r="B93" s="4">
+        <v>77.8</v>
+      </c>
+      <c r="C93" s="4">
+        <v>45.533999999999999</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A94" s="4">
+        <v>0.92</v>
+      </c>
+      <c r="B94" s="4">
+        <v>77.731999999999999</v>
+      </c>
+      <c r="C94" s="4">
+        <v>45.497</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A95" s="4">
+        <v>0.93</v>
+      </c>
+      <c r="B95" s="4">
+        <v>77.664000000000001</v>
+      </c>
+      <c r="C95" s="4">
+        <v>45.459000000000003</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A96" s="4">
+        <v>0.94</v>
+      </c>
+      <c r="B96" s="4">
+        <v>77.596999999999994</v>
+      </c>
+      <c r="C96" s="4">
+        <v>45.421999999999997</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A97" s="4">
+        <v>0.95</v>
+      </c>
+      <c r="B97" s="4">
+        <v>77.531000000000006</v>
+      </c>
+      <c r="C97" s="4">
+        <v>45.386000000000003</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A98" s="4">
+        <v>0.96</v>
+      </c>
+      <c r="B98" s="4">
+        <v>77.465000000000003</v>
+      </c>
+      <c r="C98" s="4">
+        <v>45.35</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A99" s="4">
+        <v>0.97</v>
+      </c>
+      <c r="B99" s="4">
+        <v>77.400000000000006</v>
+      </c>
+      <c r="C99" s="4">
+        <v>45.314</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A100" s="4">
+        <v>0.98</v>
+      </c>
+      <c r="B100" s="4">
+        <v>77.335999999999999</v>
+      </c>
+      <c r="C100" s="4">
+        <v>45.277999999999999</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A101" s="4">
+        <v>0.99</v>
+      </c>
+      <c r="B101" s="4">
+        <v>77.272000000000006</v>
+      </c>
+      <c r="C101" s="4">
+        <v>45.243000000000002</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A102" s="4">
+        <v>1</v>
+      </c>
+      <c r="B102" s="4">
+        <v>77.207999999999998</v>
+      </c>
+      <c r="C102" s="4">
+        <v>45.207999999999998</v>
+      </c>
+    </row>
+    <row r="138" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H138">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>